<commit_message>
docs(notebooks): update quickstart and existing notebooks
Refresh outputs and minor edits across notebooks 01-09 and
regenerated output files (JSON, XLSX, ZIP).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notebooks/output/tc99m_results.xlsx
+++ b/notebooks/output/tc99m_results.xlsx
@@ -586,10 +586,10 @@
     <t>Y-86m</t>
   </si>
   <si>
+    <t>Y-87</t>
+  </si>
+  <si>
     <t>Y-87m</t>
-  </si>
-  <si>
-    <t>Y-87</t>
   </si>
   <si>
     <t>Mo-94</t>
@@ -3750,7 +3750,7 @@
         <v>1.069920002376643E-08</v>
       </c>
       <c r="H52" s="3">
-        <v>9.649373096996609E-11</v>
+        <v>9.649373097182617E-11</v>
       </c>
       <c r="I52" s="3">
         <v>7.132800015844288E-11</v>
@@ -3798,7 +3798,7 @@
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3">
-        <v>0.6605236943840167</v>
+        <v>0.6622380139841406</v>
       </c>
       <c r="H53" s="3">
         <v>0</v>
@@ -3851,13 +3851,13 @@
         <v>0.82</v>
       </c>
       <c r="G54" s="3">
-        <v>0.1152886195489359</v>
+        <v>0.1156265627537979</v>
       </c>
       <c r="H54" s="3">
         <v>0</v>
       </c>
       <c r="I54" s="3">
-        <v>0.0007685907969929063</v>
+        <v>0.0007708437516919859</v>
       </c>
       <c r="J54" s="3">
         <v>16</v>
@@ -4314,13 +4314,13 @@
         <v>5532360</v>
       </c>
       <c r="G63" s="3">
-        <v>2.246493714552107E-06</v>
+        <v>2.252286590733003E-06</v>
       </c>
       <c r="H63" s="3">
-        <v>2.392677846086431E-08</v>
+        <v>2.398847677087512E-08</v>
       </c>
       <c r="I63" s="3">
-        <v>1.497662476368071E-08</v>
+        <v>1.501524393822002E-08</v>
       </c>
       <c r="J63" s="3">
         <v>16</v>
@@ -4341,7 +4341,7 @@
         <v>72</v>
       </c>
       <c r="P63" s="3">
-        <v>2.392677846133227E-08</v>
+        <v>2.398847677107443E-08</v>
       </c>
       <c r="Q63" s="3">
         <v>0</v>
@@ -4365,13 +4365,13 @@
         <v>1.23075E+27</v>
       </c>
       <c r="G64" s="3">
-        <v>210.5633419233672</v>
+        <v>210.9855317414799</v>
       </c>
       <c r="H64" s="3">
-        <v>1.024594744494509E-20</v>
+        <v>1.026649107173658E-20</v>
       </c>
       <c r="I64" s="3">
-        <v>1.403755612822448</v>
+        <v>1.406570211609866</v>
       </c>
       <c r="J64" s="3">
         <v>16</v>
@@ -4395,7 +4395,7 @@
         <v>0</v>
       </c>
       <c r="Q64" s="3">
-        <v>1.024594744494509E-20</v>
+        <v>1.026649107173658E-20</v>
       </c>
     </row>
     <row r="65" spans="1:17">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="F82" s="3"/>
       <c r="G82" s="3">
-        <v>38.69771589997226</v>
+        <v>38.83767227160691</v>
       </c>
       <c r="H82" s="3">
         <v>0</v>
@@ -5342,13 +5342,13 @@
         <v>84060</v>
       </c>
       <c r="G83" s="3">
-        <v>376847799.2913398</v>
+        <v>377620230.7649989</v>
       </c>
       <c r="H83" s="3">
-        <v>94177543.08436212</v>
+        <v>94370580.42989156</v>
       </c>
       <c r="I83" s="3">
-        <v>2512318.661942265</v>
+        <v>2517468.205099992</v>
       </c>
       <c r="J83" s="3">
         <v>16</v>
@@ -5369,7 +5369,7 @@
         <v>72</v>
       </c>
       <c r="P83" s="3">
-        <v>94177543.08629604</v>
+        <v>94370580.43062586</v>
       </c>
       <c r="Q83" s="3">
         <v>0</v>
@@ -5393,7 +5393,7 @@
       </c>
       <c r="F84" s="3"/>
       <c r="G84" s="3">
-        <v>4189415644.815259</v>
+        <v>4191636196.542623</v>
       </c>
       <c r="H84" s="3">
         <v>0</v>
@@ -5444,7 +5444,7 @@
       </c>
       <c r="F85" s="3"/>
       <c r="G85" s="3">
-        <v>0.08813584371215752</v>
+        <v>0.0884532342505587</v>
       </c>
       <c r="H85" s="3">
         <v>0</v>
@@ -5497,13 +5497,13 @@
         <v>3078</v>
       </c>
       <c r="G86" s="3">
-        <v>0.21444020009968</v>
+        <v>0.2152128207113262</v>
       </c>
       <c r="H86" s="3">
-        <v>7.609242268113925E-10</v>
+        <v>7.636658104565245E-10</v>
       </c>
       <c r="I86" s="3">
-        <v>0.001429601333997866</v>
+        <v>0.001434752138075508</v>
       </c>
       <c r="J86" s="3">
         <v>16</v>
@@ -5524,7 +5524,7 @@
         <v>72</v>
       </c>
       <c r="P86" s="3">
-        <v>7.609242268442884E-10</v>
+        <v>7.636658104712742E-10</v>
       </c>
       <c r="Q86" s="3">
         <v>0</v>
@@ -5548,7 +5548,7 @@
       </c>
       <c r="F87" s="3"/>
       <c r="G87" s="3">
-        <v>0.03721200843585283</v>
+        <v>0.0372871622807306</v>
       </c>
       <c r="H87" s="3">
         <v>0</v>
@@ -5601,13 +5601,13 @@
         <v>156</v>
       </c>
       <c r="G88" s="3">
-        <v>0.007967640108572817</v>
+        <v>0.007986407648589463</v>
       </c>
       <c r="H88" s="3">
-        <v>1.503226482994294E-169</v>
+        <v>1.506767288439297E-169</v>
       </c>
       <c r="I88" s="3">
-        <v>5.311760072381878E-05</v>
+        <v>5.324271765726309E-05</v>
       </c>
       <c r="J88" s="3">
         <v>16</v>
@@ -5628,7 +5628,7 @@
         <v>72</v>
       </c>
       <c r="P88" s="3">
-        <v>1.503226483052666E-169</v>
+        <v>1.506767288459328E-169</v>
       </c>
       <c r="Q88" s="3">
         <v>0</v>
@@ -6013,13 +6013,13 @@
         <v>3.1242E+26</v>
       </c>
       <c r="G96" s="3">
-        <v>150230943332.4394</v>
+        <v>150224463565.2912</v>
       </c>
       <c r="H96" s="3">
-        <v>2.879783040420835E-11</v>
+        <v>2.879658829534125E-11</v>
       </c>
       <c r="I96" s="3">
-        <v>1001539622.216263</v>
+        <v>1001496423.768608</v>
       </c>
       <c r="J96" s="3">
         <v>16</v>
@@ -6043,7 +6043,7 @@
         <v>0</v>
       </c>
       <c r="Q96" s="3">
-        <v>2.879783040420835E-11</v>
+        <v>2.879658829534125E-11</v>
       </c>
     </row>
     <row r="97" spans="1:17">
@@ -6841,7 +6841,7 @@
       </c>
       <c r="F112" s="3"/>
       <c r="G112" s="3">
-        <v>751718805954.8778</v>
+        <v>751651017256.4495</v>
       </c>
       <c r="H112" s="3">
         <v>0</v>
@@ -6892,13 +6892,13 @@
         <v>15.8</v>
       </c>
       <c r="G113" s="3">
-        <v>77939074306.7384</v>
+        <v>77972470832.6387</v>
       </c>
       <c r="H113" s="3">
         <v>0</v>
       </c>
       <c r="I113" s="3">
-        <v>519593828.7115893</v>
+        <v>519816472.2175913</v>
       </c>
       <c r="J113" s="3">
         <v>16</v>
@@ -6943,13 +6943,13 @@
         <v>852</v>
       </c>
       <c r="G114" s="3">
-        <v>1166400877.333632</v>
+        <v>1166232356.739933</v>
       </c>
       <c r="H114" s="3">
-        <v>3.466269787764098E-22</v>
+        <v>3.465768984179105E-22</v>
       </c>
       <c r="I114" s="3">
-        <v>7776005.848890883</v>
+        <v>7774882.378266217</v>
       </c>
       <c r="J114" s="3">
         <v>16</v>
@@ -6970,7 +6970,7 @@
         <v>72</v>
       </c>
       <c r="P114" s="3">
-        <v>3.466269787927032E-22</v>
+        <v>3.465768984254867E-22</v>
       </c>
       <c r="Q114" s="3">
         <v>0</v>
@@ -7757,13 +7757,13 @@
         <v>36648</v>
       </c>
       <c r="G130" s="3">
-        <v>0.7758125614603597</v>
+        <v>0.7778648247809754</v>
       </c>
       <c r="H130" s="3">
-        <v>0.1399464184556316</v>
+        <v>0.1403217977520069</v>
       </c>
       <c r="I130" s="3">
-        <v>0.005172083743069065</v>
+        <v>0.005185765498539836</v>
       </c>
       <c r="J130" s="3">
         <v>16</v>
@@ -7784,10 +7784,10 @@
         <v>72</v>
       </c>
       <c r="P130" s="3">
-        <v>0.1218401202719896</v>
+        <v>0.1221624249396827</v>
       </c>
       <c r="Q130" s="3">
-        <v>0.018106298183642</v>
+        <v>0.0181593728123242</v>
       </c>
     </row>
     <row r="131" spans="1:17">
@@ -7963,13 +7963,13 @@
         <v>311760</v>
       </c>
       <c r="G134" s="3">
-        <v>2.508808818564925</v>
+        <v>2.517894781096592</v>
       </c>
       <c r="H134" s="3">
-        <v>0.3618382115152144</v>
+        <v>0.3631486535140073</v>
       </c>
       <c r="I134" s="3">
-        <v>0.01672539212376617</v>
+        <v>0.01678596520731062</v>
       </c>
       <c r="J134" s="3">
         <v>16</v>
@@ -7990,10 +7990,10 @@
         <v>72</v>
       </c>
       <c r="P134" s="3">
-        <v>0.3618382114534961</v>
+        <v>0.3631486534479054</v>
       </c>
       <c r="Q134" s="3">
-        <v>6.171835265078585E-11</v>
+        <v>6.610190173006458E-11</v>
       </c>
     </row>
     <row r="135" spans="1:17">
@@ -8016,13 +8016,13 @@
         <v>52.7</v>
       </c>
       <c r="G135" s="3">
-        <v>979282666.2080213</v>
+        <v>979717036.017977</v>
       </c>
       <c r="H135" s="3">
         <v>0</v>
       </c>
       <c r="I135" s="3">
-        <v>6528551.108053476</v>
+        <v>6531446.906786514</v>
       </c>
       <c r="J135" s="3">
         <v>16</v>
@@ -8067,13 +8067,13 @@
         <v>2.86</v>
       </c>
       <c r="G136" s="3">
-        <v>0.3025755654763828</v>
+        <v>0.3036655748579766</v>
       </c>
       <c r="H136" s="3">
         <v>0</v>
       </c>
       <c r="I136" s="3">
-        <v>0.002017170436509219</v>
+        <v>0.002024437165719844</v>
       </c>
       <c r="J136" s="3">
         <v>16</v>
@@ -8271,13 +8271,13 @@
         <v>15</v>
       </c>
       <c r="G140" s="3">
-        <v>0.04517970368234782</v>
+        <v>0.04527362530789504</v>
       </c>
       <c r="H140" s="3">
-        <v>3.326288387902275E-171</v>
+        <v>3.33412336165292E-171</v>
       </c>
       <c r="I140" s="3">
-        <v>0.0003011980245489855</v>
+        <v>0.0003018241687193003</v>
       </c>
       <c r="J140" s="3">
         <v>16</v>
@@ -8301,7 +8301,7 @@
         <v>0</v>
       </c>
       <c r="Q140" s="3">
-        <v>3.326288387902275E-171</v>
+        <v>3.33412336165292E-171</v>
       </c>
     </row>
     <row r="141" spans="1:17">
@@ -9384,7 +9384,7 @@
         <v>0</v>
       </c>
       <c r="H162" s="3">
-        <v>9.990749496260979E-10</v>
+        <v>1.001754774831585E-09</v>
       </c>
       <c r="I162" s="3">
         <v>0</v>
@@ -9411,7 +9411,7 @@
         <v>0</v>
       </c>
       <c r="Q162" s="3">
-        <v>9.990749496260979E-10</v>
+        <v>1.001754774831585E-09</v>
       </c>
     </row>
     <row r="163" spans="1:17">
@@ -9532,13 +9532,13 @@
         <v>3023220</v>
       </c>
       <c r="G165" s="3">
-        <v>41.20644359980112</v>
+        <v>41.35548564007702</v>
       </c>
       <c r="H165" s="3">
-        <v>0.8038909332531287</v>
+        <v>0.8067986279239511</v>
       </c>
       <c r="I165" s="3">
-        <v>0.2747096239986741</v>
+        <v>0.2757032376005135</v>
       </c>
       <c r="J165" s="3">
         <v>16</v>
@@ -9559,10 +9559,10 @@
         <v>72</v>
       </c>
       <c r="P165" s="3">
-        <v>0.7923865073724354</v>
+        <v>0.7952525373286449</v>
       </c>
       <c r="Q165" s="3">
-        <v>0.01150442588069323</v>
+        <v>0.0115460905953062</v>
       </c>
     </row>
     <row r="166" spans="1:17">
@@ -9583,13 +9583,13 @@
         <v>4326</v>
       </c>
       <c r="G166" s="3">
-        <v>5168697950.931241</v>
+        <v>5171352872.131046</v>
       </c>
       <c r="H166" s="3">
-        <v>5988.730613855321</v>
+        <v>5991.739191779136</v>
       </c>
       <c r="I166" s="3">
-        <v>34457986.33954161</v>
+        <v>34475685.81420697</v>
       </c>
       <c r="J166" s="3">
         <v>16</v>
@@ -9610,10 +9610,10 @@
         <v>72</v>
       </c>
       <c r="P166" s="3">
-        <v>5024.94328850696</v>
+        <v>5027.52436958214</v>
       </c>
       <c r="Q166" s="3">
-        <v>963.7873253483613</v>
+        <v>964.2148221969956</v>
       </c>
     </row>
     <row r="167" spans="1:17">
@@ -9634,13 +9634,13 @@
         <v>3.15576E+21</v>
       </c>
       <c r="G167" s="3">
-        <v>63119105.73301613</v>
+        <v>63215291.1121275</v>
       </c>
       <c r="H167" s="3">
-        <v>1.197832458203775E-09</v>
+        <v>1.199657800465895E-09</v>
       </c>
       <c r="I167" s="3">
-        <v>420794.0382201075</v>
+        <v>421435.27408085</v>
       </c>
       <c r="J167" s="3">
         <v>16</v>
@@ -9664,7 +9664,7 @@
         <v>0</v>
       </c>
       <c r="Q167" s="3">
-        <v>1.197832458203775E-09</v>
+        <v>1.199657800465895E-09</v>
       </c>
     </row>
     <row r="168" spans="1:17">
@@ -9733,11 +9733,9 @@
       <c r="D169" s="1">
         <v>87</v>
       </c>
-      <c r="E169" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="E169" s="2"/>
       <c r="F169" s="3">
-        <v>48132</v>
+        <v>287280</v>
       </c>
       <c r="G169" s="3">
         <v>0</v>
@@ -9786,9 +9784,11 @@
       <c r="D170" s="1">
         <v>87</v>
       </c>
-      <c r="E170" s="2"/>
+      <c r="E170" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="F170" s="3">
-        <v>287280</v>
+        <v>48132</v>
       </c>
       <c r="G170" s="3">
         <v>0</v>
@@ -9891,13 +9891,13 @@
         <v>237384</v>
       </c>
       <c r="G172" s="3">
-        <v>29385712306.96463</v>
+        <v>29400157670.90543</v>
       </c>
       <c r="H172" s="3">
-        <v>5091286190.871343</v>
+        <v>5093788954.219334</v>
       </c>
       <c r="I172" s="3">
-        <v>195904748.7130975</v>
+        <v>196001051.1393695</v>
       </c>
       <c r="J172" s="3">
         <v>16</v>
@@ -9918,7 +9918,7 @@
         <v>72</v>
       </c>
       <c r="P172" s="3">
-        <v>5091286190.953646</v>
+        <v>5093788954.241697</v>
       </c>
       <c r="Q172" s="3">
         <v>0</v>
@@ -10450,7 +10450,7 @@
       <c r="E183" s="2"/>
       <c r="F183" s="3"/>
       <c r="G183" s="3">
-        <v>1.836969112932438E-05</v>
+        <v>1.866069169712705E-05</v>
       </c>
       <c r="H183" s="3">
         <v>0</v>
@@ -10603,13 +10603,13 @@
         <v>21636</v>
       </c>
       <c r="G186" s="3">
-        <v>276690168923.4486</v>
+        <v>276655343704.1462</v>
       </c>
       <c r="H186" s="3">
-        <v>21062540887.7324</v>
+        <v>21062841425.04351</v>
       </c>
       <c r="I186" s="3">
-        <v>1844601126.156324</v>
+        <v>1844368958.027641</v>
       </c>
       <c r="J186" s="3">
         <v>16</v>
@@ -10630,10 +10630,10 @@
         <v>72</v>
       </c>
       <c r="P186" s="3">
-        <v>16282258746.29516</v>
+        <v>16280209402.67813</v>
       </c>
       <c r="Q186" s="3">
-        <v>4780282141.437244</v>
+        <v>4782632022.365381</v>
       </c>
     </row>
     <row r="187" spans="1:17">
@@ -10814,7 +10814,7 @@
         <v>0</v>
       </c>
       <c r="H190" s="3">
-        <v>1.200747287898958E-13</v>
+        <v>1.203968059707482E-13</v>
       </c>
       <c r="I190" s="3">
         <v>0</v>
@@ -10841,7 +10841,7 @@
         <v>0</v>
       </c>
       <c r="Q190" s="3">
-        <v>1.200747287898958E-13</v>
+        <v>1.203968059707482E-13</v>
       </c>
     </row>
     <row r="191" spans="1:17">
@@ -11064,13 +11064,13 @@
         <v>6753180000000</v>
       </c>
       <c r="G195" s="3">
-        <v>990550374075.6962</v>
+        <v>990464502954.453</v>
       </c>
       <c r="H195" s="3">
-        <v>11252.08133038965</v>
+        <v>11251.0501571549</v>
       </c>
       <c r="I195" s="3">
-        <v>6603669160.504642</v>
+        <v>6603096686.36302</v>
       </c>
       <c r="J195" s="3">
         <v>16</v>
@@ -11091,10 +11091,10 @@
         <v>72</v>
       </c>
       <c r="P195" s="3">
-        <v>8784.305664778125</v>
+        <v>8783.544150577012</v>
       </c>
       <c r="Q195" s="3">
-        <v>2467.775665611529</v>
+        <v>2467.506006577883</v>
       </c>
     </row>
     <row r="196" spans="1:17">

</xml_diff>